<commit_message>
Add MAPE metric, discussion writeups, and input range validation for the web predictor
</commit_message>
<xml_diff>
--- a/Results_Summary_Tuned200.xlsx
+++ b/Results_Summary_Tuned200.xlsx
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,15 +796,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>MAPE</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>IoA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Theta Mean</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Theta CoV</t>
         </is>
@@ -838,15 +843,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>6.988 ± 2.359</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>0.979 ± 0.017</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>1.004 ± 0.033</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>0.108 ± 0.036</t>
         </is>
@@ -880,15 +890,20 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>7.771 ± 2.454</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>0.976 ± 0.017</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>0.989 ± 0.021</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>0.108 ± 0.037</t>
         </is>
@@ -922,15 +937,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>9.023 ± 2.227</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>0.973 ± 0.020</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>0.994 ± 0.046</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>0.119 ± 0.035</t>
         </is>
@@ -964,15 +984,20 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>10.326 ± 3.106</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>0.965 ± 0.018</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>0.989 ± 0.032</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>0.133 ± 0.041</t>
         </is>
@@ -989,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1020,15 +1045,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>MAPE</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>IoA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Theta Mean</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Theta CoV</t>
         </is>
@@ -1062,15 +1092,20 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>8.552 ± 2.292</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>0.970 ± 0.019</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>1.014 ± 0.049</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>0.161 ± 0.128</t>
         </is>
@@ -1104,15 +1139,20 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>9.242 ± 2.717</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>0.964 ± 0.019</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>0.988 ± 0.029</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>0.128 ± 0.029</t>
         </is>
@@ -1146,15 +1186,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>10.165 ± 2.297</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>0.962 ± 0.019</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>0.993 ± 0.029</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>0.132 ± 0.025</t>
         </is>
@@ -1188,15 +1233,20 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>10.937 ± 2.228</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>0.957 ± 0.020</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>0.991 ± 0.030</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>0.142 ± 0.027</t>
         </is>

</xml_diff>